<commit_message>
change csv file: for git commit (year/ month)
</commit_message>
<xml_diff>
--- a/StateOfPractice/DomainMeasurements/InverseKinematics-Ryan/summary.xlsx
+++ b/StateOfPractice/DomainMeasurements/InverseKinematics-Ryan/summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\coding\AIMSS\StateOfPractice\DomainMeasurements\InverseKinematics-Ryan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC80BCA-11BB-4FD2-8948-913900E36316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C5BCBC-144C-403C-9661-51CFCF486BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="appendix-B-wide-summary" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2104" uniqueCount="691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2104" uniqueCount="675">
   <si>
     <t>Metric
 指标（见附录 A 与附录 B）</t>
@@ -1425,84 +1425,6 @@
     <t>Doxygen,automated testing</t>
   </si>
   <si>
-    <t>Is there evidence of continuous integration? (for example mentioned in documentation, Jenkins, Travis CI, Bamboo, other) (yes∗, no, unclear)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/bazel.yml, .github/workflows/ci.yml, .github/workflows/docker-nightly.yml, .github/workflows/package_xml.yml, .github/workflows/pr-collection-labeler.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/sync_protected_branches.yml, .github/workflows/test_suite_linux.yml, .github/workflows/test_suite_linux_develop.yml, .github/workflows/test_suite_mac.yml, .github/workflows/test_suite_mac_develop.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/cmake.yml, appveyor.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/build.yml, .github/workflows/build_steps.sh, .github/workflows/lint.yml, .github/workflows/live.yml, .github/workflows/publish-wasm.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/mirror-rolling-to-master.yaml, .github/workflows/pr.yaml, .github/workflows/release-nightlies.yaml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/ci.yaml, .travis.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/clang_format.yml, .github/workflows/test_docs.yml, .github/workflows/test_macos.yml, .github/workflows/test_ubuntu.yml, .github/workflows/test_windows.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/stale.yml, .jenkins/Jenkinsfile-experimental, .jenkins/Jenkinsfile-external-examples, .jenkins/Jenkinsfile-production, .jenkins/Jenkinsfile-staging)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/cancel_branch_jobs.yml, .github/workflows/ci_altlinux.yml, .github/workflows/ci_freebsd.yml, .github/workflows/ci_gz_physics.yml, .github/workflows/ci_lint.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/_ci-ubuntu.yml, .github/workflows/ue4_content.yml, .github/workflows/ue4_dev.yml, .github/workflows/ue4_release.yml, .github/workflows/ue5_dev.yml)</t>
-  </si>
-  <si>
-    <t>yes (.travis.yml, appveyor.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/continuous_integration.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/before_all.sh, .github/workflows/before_build.sh, .github/workflows/before_build_windows.ps1, .github/workflows/build.yml, .github/workflows/format.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/check-changelog.yml, .github/workflows/check_label.yml, .github/workflows/cmake/linux-debug-toolchain.cmake, .github/workflows/dockgen.yml, .github/workflows/linux.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/main.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/build-and-test.yml, .github/workflows/ci-macos-linux-windows-pixi.yml, .github/workflows/launch-conda-packages-build.yml, .github/workflows/launch-perf-test.yml, .github/workflows/nightly-generate-binaries.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/ci.yaml, .github/workflows/docker.yaml, .github/workflows/docker_lint.yaml, .github/workflows/format.yaml, .github/workflows/prerelease.yaml)</t>
-  </si>
-  <si>
-    <t>yes (.travis.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/install_and_test.yml)</t>
-  </si>
-  <si>
-    <t>yes (appveyor.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/clang_format.yml, .github/workflows/cpp_unittests.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/build-linux.yml, .github/workflows/build-macos.yml, .github/workflows/build-windows.yml, .github/workflows/check-clang-format.yml, appveyor.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/build.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/ci.yml, .github/workflows/docker-build.yml, .github/workflows/nightly-merge.yml, .github/workflows/pr-commands.yml, .github/workflows/python.yml)</t>
-  </si>
-  <si>
-    <t>yes (.github/workflows/openrtm_linux.yml, azure-pipelines.yml)</t>
-  </si>
-  <si>
     <t>gz-sim10_10.0.0</t>
   </si>
   <si>
@@ -2033,168 +1955,9 @@
     <t>Numbers of commits by year in the last 5 years. (Count from as early as possible if the project is younger than 5 years.) (list of numbers)</t>
   </si>
   <si>
-    <t>2022: 475; 2023: 321; 2024: 290; 2025: 250; 2026: 81</t>
-  </si>
-  <si>
-    <t>2022: 1027; 2023: 608; 2024: 221; 2025: 53; 2026: 16</t>
-  </si>
-  <si>
-    <t>2022: 152; 2023: 8; 2024: 6; 2025: 5; 2026: 0</t>
-  </si>
-  <si>
-    <t>2022: 158; 2023: 251; 2024: 163; 2025: 166; 2026: 165</t>
-  </si>
-  <si>
-    <t>2022: 491; 2023: 840; 2024: 1244; 2025: 1315; 2026: 781</t>
-  </si>
-  <si>
-    <t>2022: 6; 2023: 9; 2024: 8; 2025: 10; 2026: 5</t>
-  </si>
-  <si>
-    <t>2022: 12; 2023: 9; 2024: 13; 2025: 31; 2026: 14</t>
-  </si>
-  <si>
-    <t>2022: 683; 2023: 889; 2024: 383; 2025: 0; 2026: 0</t>
-  </si>
-  <si>
-    <t>2022: 6; 2023: 8; 2024: 9; 2025: 14; 2026: 3</t>
-  </si>
-  <si>
-    <t>2022: 238; 2023: 0; 2024: 0; 2025: 1; 2026: 1</t>
-  </si>
-  <si>
-    <t>2022: 1713; 2023: 1618; 2024: 1247; 2025: 1251; 2026: 481</t>
-  </si>
-  <si>
-    <t>2022: 43; 2023: 7; 2024: 291; 2025: 394; 2026: 257</t>
-  </si>
-  <si>
-    <t>2022: 385; 2023: 269; 2024: 471; 2025: 113; 2026: 35</t>
-  </si>
-  <si>
-    <t>2022: 1; 2023: 0; 2024: 0; 2025: 0; 2026: 0</t>
-  </si>
-  <si>
-    <t>2022: 48; 2023: 13; 2024: 45; 2025: 25; 2026: 6</t>
-  </si>
-  <si>
-    <t>2022: 30; 2023: 68; 2024: 23; 2025: 298; 2026: 200</t>
-  </si>
-  <si>
-    <t>2022: 898; 2023: 556; 2024: 1743; 2025: 2343; 2026: 843</t>
-  </si>
-  <si>
-    <t>2022: 48; 2023: 14; 2024: 12; 2025: 22; 2026: 2</t>
-  </si>
-  <si>
-    <t>2022: 840; 2023: 409; 2024: 389; 2025: 338; 2026: 188</t>
-  </si>
-  <si>
-    <t>2022: 476; 2023: 331; 2024: 193; 2025: 117; 2026: 5</t>
-  </si>
-  <si>
-    <t>2022: 0; 2023: 0; 2024: 0; 2025: 0; 2026: 0</t>
-  </si>
-  <si>
-    <t>2022: 225; 2023: 162; 2024: 99; 2025: 19; 2026: 25</t>
-  </si>
-  <si>
-    <t>2022: 1216; 2023: 1294; 2024: 1386; 2025: 1236; 2026: 604</t>
-  </si>
-  <si>
-    <t>2022: 0; 2023: 1; 2024: 0; 2025: 0; 2026: 0</t>
-  </si>
-  <si>
-    <t>2022: 514; 2023: 437; 2024: 346; 2025: 130; 2026: 299</t>
-  </si>
-  <si>
-    <t>2022: 1774; 2023: 1441; 2024: 1193; 2025: 2722; 2026: 1141</t>
-  </si>
-  <si>
-    <t>2022: 336; 2023: 508; 2024: 262; 2025: 442; 2026: 82</t>
-  </si>
-  <si>
-    <t>2022: 221; 2023: 59; 2024: 69; 2025: 72; 2026: 40</t>
-  </si>
-  <si>
     <t>Numbers of commits by month in the last 12 months. (list of numbers)</t>
   </si>
   <si>
-    <t>2025-06: 15; 2025-07: 24; 2025-08: 40; 2025-09: 17; 2025-10: 16; 2025-11: 21; 2025-12: 11; 2026-01: 17; 2026-02: 27; 2026-03: 19; 2026-04: 9; 2026-05: 9</t>
-  </si>
-  <si>
-    <t>2025-06: 4; 2025-07: 9; 2025-08: 10; 2025-09: 0; 2025-10: 0; 2025-11: 2; 2025-12: 0; 2026-01: 0; 2026-02: 9; 2026-03: 3; 2026-04: 3; 2026-05: 1</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 0; 2025-08: 0; 2025-09: 0; 2025-10: 1; 2025-11: 0; 2025-12: 0; 2026-01: 0; 2026-02: 0; 2026-03: 0; 2026-04: 0; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 21; 2025-07: 19; 2025-08: 1; 2025-09: 8; 2025-10: 12; 2025-11: 39; 2025-12: 16; 2026-01: 8; 2026-02: 32; 2026-03: 43; 2026-04: 66; 2026-05: 16</t>
-  </si>
-  <si>
-    <t>2025-06: 74; 2025-07: 138; 2025-08: 111; 2025-09: 88; 2025-10: 140; 2025-11: 176; 2025-12: 115; 2026-01: 144; 2026-02: 203; 2026-03: 183; 2026-04: 177; 2026-05: 74</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 0; 2025-08: 0; 2025-09: 0; 2025-10: 0; 2025-11: 0; 2025-12: 0; 2026-01: 1; 2026-02: 0; 2026-03: 3; 2026-04: 1; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 3; 2025-07: 2; 2025-08: 0; 2025-09: 2; 2025-10: 7; 2025-11: 1; 2025-12: 4; 2026-01: 2; 2026-02: 1; 2026-03: 2; 2026-04: 9; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 0; 2025-08: 0; 2025-09: 0; 2025-10: 0; 2025-11: 0; 2025-12: 0; 2026-01: 0; 2026-02: 0; 2026-03: 0; 2026-04: 0; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 1; 2025-08: 0; 2025-09: 1; 2025-10: 2; 2025-11: 0; 2025-12: 0; 2026-01: 0; 2026-02: 0; 2026-03: 2; 2026-04: 1; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 0; 2025-08: 0; 2025-09: 0; 2025-10: 0; 2025-11: 0; 2025-12: 0; 2026-01: 0; 2026-02: 0; 2026-03: 1; 2026-04: 0; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 82; 2025-07: 84; 2025-08: 80; 2025-09: 131; 2025-10: 162; 2025-11: 79; 2025-12: 79; 2026-01: 76; 2026-02: 102; 2026-03: 119; 2026-04: 150; 2026-05: 34</t>
-  </si>
-  <si>
-    <t>2025-06: 4; 2025-07: 8; 2025-08: 22; 2025-09: 4; 2025-10: 44; 2025-11: 199; 2025-12: 63; 2026-01: 140; 2026-02: 19; 2026-03: 4; 2026-04: 5; 2026-05: 89</t>
-  </si>
-  <si>
-    <t>2025-06: 7; 2025-07: 1; 2025-08: 16; 2025-09: 5; 2025-10: 18; 2025-11: 18; 2025-12: 2; 2026-01: 3; 2026-02: 2; 2026-03: 6; 2026-04: 20; 2026-05: 4</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 3; 2025-08: 5; 2025-09: 0; 2025-10: 2; 2025-11: 1; 2025-12: 0; 2026-01: 2; 2026-02: 3; 2026-03: 1; 2026-04: 0; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 28; 2025-07: 0; 2025-08: 54; 2025-09: 3; 2025-10: 12; 2025-11: 0; 2025-12: 124; 2026-01: 41; 2026-02: 22; 2026-03: 83; 2026-04: 47; 2026-05: 7</t>
-  </si>
-  <si>
-    <t>2025-06: 90; 2025-07: 141; 2025-08: 49; 2025-09: 87; 2025-10: 108; 2025-11: 167; 2025-12: 302; 2026-01: 155; 2026-02: 280; 2026-03: 248; 2026-04: 154; 2026-05: 6</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 1; 2025-08: 3; 2025-09: 1; 2025-10: 6; 2025-11: 1; 2025-12: 6; 2026-01: 0; 2026-02: 1; 2026-03: 0; 2026-04: 0; 2026-05: 1</t>
-  </si>
-  <si>
-    <t>2025-06: 24; 2025-07: 30; 2025-08: 10; 2025-09: 25; 2025-10: 25; 2025-11: 25; 2025-12: 33; 2026-01: 34; 2026-02: 45; 2026-03: 83; 2026-04: 19; 2026-05: 7</t>
-  </si>
-  <si>
-    <t>2025-06: 9; 2025-07: 2; 2025-08: 1; 2025-09: 1; 2025-10: 5; 2025-11: 18; 2025-12: 14; 2026-01: 1; 2026-02: 0; 2026-03: 4; 2026-04: 0; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 0; 2025-08: 0; 2025-09: 0; 2025-10: 0; 2025-11: 0; 2025-12: 0; 2026-01: 3; 2026-02: 20; 2026-03: 0; 2026-04: 0; 2026-05: 2</t>
-  </si>
-  <si>
-    <t>2025-06: 52; 2025-07: 72; 2025-08: 93; 2025-09: 140; 2025-10: 155; 2025-11: 103; 2025-12: 103; 2026-01: 139; 2026-02: 134; 2026-03: 178; 2026-04: 104; 2026-05: 49</t>
-  </si>
-  <si>
-    <t>2025-06: 0; 2025-07: 1; 2025-08: 10; 2025-09: 5; 2025-10: 9; 2025-11: 21; 2025-12: 26; 2026-01: 73; 2026-02: 81; 2026-03: 100; 2026-04: 39; 2026-05: 6</t>
-  </si>
-  <si>
-    <t>2025-06: 339; 2025-07: 273; 2025-08: 204; 2025-09: 380; 2025-10: 284; 2025-11: 290; 2025-12: 242; 2026-01: 221; 2026-02: 199; 2026-03: 350; 2026-04: 300; 2026-05: 71</t>
-  </si>
-  <si>
-    <t>2025-06: 27; 2025-07: 57; 2025-08: 57; 2025-09: 27; 2025-10: 14; 2025-11: 33; 2025-12: 20; 2026-01: 36; 2026-02: 25; 2026-03: 13; 2026-04: 8; 2026-05: 0</t>
-  </si>
-  <si>
-    <t>2025-06: 4; 2025-07: 6; 2025-08: 0; 2025-09: 18; 2025-10: 10; 2025-11: 7; 2025-12: 6; 2026-01: 0; 2026-02: 0; 2026-03: 26; 2026-04: 9; 2026-05: 5</t>
-  </si>
-  <si>
     <t>Number of code lines in text-based files. (number)</t>
   </si>
   <si>
@@ -2217,13 +1980,225 @@
   </si>
   <si>
     <t>Number of closed pull requests. (number)</t>
+  </si>
+  <si>
+    <t>[475, 321, 290, 250, 81]</t>
+  </si>
+  <si>
+    <t>[1027, 608, 221, 53, 16]</t>
+  </si>
+  <si>
+    <t>[152, 8, 6, 5, 0]</t>
+  </si>
+  <si>
+    <t>[158, 251, 163, 166, 165]</t>
+  </si>
+  <si>
+    <t>[491, 840, 1244, 1315, 781]</t>
+  </si>
+  <si>
+    <t>[6, 9, 8, 10, 5]</t>
+  </si>
+  <si>
+    <t>[12, 9, 13, 31, 14]</t>
+  </si>
+  <si>
+    <t>[683, 889, 383, 0, 0]</t>
+  </si>
+  <si>
+    <t>[6, 8, 9, 14, 3]</t>
+  </si>
+  <si>
+    <t>[238, 0, 0, 1, 1]</t>
+  </si>
+  <si>
+    <t>[1713, 1618, 1247, 1251, 481]</t>
+  </si>
+  <si>
+    <t>[43, 7, 291, 394, 257]</t>
+  </si>
+  <si>
+    <t>[385, 269, 471, 113, 35]</t>
+  </si>
+  <si>
+    <t>[1, 0, 0, 0, 0]</t>
+  </si>
+  <si>
+    <t>[48, 13, 45, 25, 6]</t>
+  </si>
+  <si>
+    <t>[30, 68, 23, 298, 201]</t>
+  </si>
+  <si>
+    <t>[898, 556, 1743, 2343, 843]</t>
+  </si>
+  <si>
+    <t>[48, 14, 12, 22, 2]</t>
+  </si>
+  <si>
+    <t>[840, 409, 389, 338, 188]</t>
+  </si>
+  <si>
+    <t>[476, 331, 193, 117, 5]</t>
+  </si>
+  <si>
+    <t>[0, 0, 0, 0, 0]</t>
+  </si>
+  <si>
+    <t>[225, 162, 99, 19, 25]</t>
+  </si>
+  <si>
+    <t>[1216, 1294, 1386, 1236, 604]</t>
+  </si>
+  <si>
+    <t>[0, 1, 0, 0, 0]</t>
+  </si>
+  <si>
+    <t>[514, 437, 346, 130, 299]</t>
+  </si>
+  <si>
+    <t>[1774, 1441, 1193, 2722, 1142]</t>
+  </si>
+  <si>
+    <t>[336, 508, 262, 442, 82]</t>
+  </si>
+  <si>
+    <t>[221, 59, 69, 72, 40]</t>
+  </si>
+  <si>
+    <t>[15, 24, 40, 17, 16, 21, 11, 17, 27, 19, 9, 9]</t>
+  </si>
+  <si>
+    <t>[4, 9, 10, 0, 0, 2, 0, 0, 9, 3, 3, 1]</t>
+  </si>
+  <si>
+    <t>[0, 0, 0, 0, 1, 0, 0, 0, 0, 0, 0, 0]</t>
+  </si>
+  <si>
+    <t>[21, 19, 1, 8, 12, 39, 16, 8, 32, 43, 66, 16]</t>
+  </si>
+  <si>
+    <t>[74, 138, 111, 88, 140, 176, 115, 144, 203, 183, 177, 74]</t>
+  </si>
+  <si>
+    <t>[0, 0, 0, 0, 0, 0, 0, 1, 0, 3, 1, 0]</t>
+  </si>
+  <si>
+    <t>[3, 2, 0, 2, 7, 1, 4, 2, 1, 2, 9, 0]</t>
+  </si>
+  <si>
+    <t>[0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0]</t>
+  </si>
+  <si>
+    <t>[0, 1, 0, 1, 2, 0, 0, 0, 0, 2, 1, 0]</t>
+  </si>
+  <si>
+    <t>[0, 0, 0, 0, 0, 0, 0, 0, 0, 1, 0, 0]</t>
+  </si>
+  <si>
+    <t>[82, 84, 80, 131, 162, 79, 79, 76, 102, 119, 150, 34]</t>
+  </si>
+  <si>
+    <t>[4, 8, 22, 4, 44, 199, 63, 140, 19, 4, 5, 89]</t>
+  </si>
+  <si>
+    <t>[7, 1, 16, 5, 18, 18, 2, 3, 2, 6, 20, 4]</t>
+  </si>
+  <si>
+    <t>[0, 3, 5, 0, 2, 1, 0, 2, 3, 1, 0, 0]</t>
+  </si>
+  <si>
+    <t>[28, 0, 54, 3, 12, 0, 124, 41, 22, 83, 47, 8]</t>
+  </si>
+  <si>
+    <t>[90, 141, 49, 87, 108, 167, 302, 155, 280, 248, 154, 6]</t>
+  </si>
+  <si>
+    <t>[0, 1, 3, 1, 6, 1, 6, 0, 1, 0, 0, 1]</t>
+  </si>
+  <si>
+    <t>[24, 30, 10, 25, 25, 25, 33, 34, 45, 83, 19, 7]</t>
+  </si>
+  <si>
+    <t>[9, 2, 1, 1, 5, 18, 14, 1, 0, 4, 0, 0]</t>
+  </si>
+  <si>
+    <t>[0, 0, 0, 0, 0, 0, 0, 3, 20, 0, 0, 2]</t>
+  </si>
+  <si>
+    <t>[52, 72, 93, 140, 155, 103, 103, 139, 134, 178, 104, 49]</t>
+  </si>
+  <si>
+    <t>[0, 1, 10, 5, 9, 21, 26, 73, 81, 100, 39, 6]</t>
+  </si>
+  <si>
+    <t>[339, 273, 204, 380, 284, 290, 242, 221, 199, 350, 300, 72]</t>
+  </si>
+  <si>
+    <t>[27, 57, 57, 27, 14, 33, 20, 36, 25, 13, 8, 0]</t>
+  </si>
+  <si>
+    <t>[4, 6, 0, 18, 10, 7, 6, 0, 0, 26, 9, 5]</t>
+  </si>
+  <si>
+    <t>yes (performance-related code or documentation references)</t>
+  </si>
+  <si>
+    <t>yes (ANN library includes performance counting macros)</t>
+  </si>
+  <si>
+    <t>yes (blast/include/extensions/authoring/NvBlastExtAuthoringFractureTool.h, blast/include/extensions/stress/NvBlastExtStressSolver.h)</t>
+  </si>
+  <si>
+    <t>yes (DART_BUILD_PROFILE, DART_PROFILE_TRACY, DART_ENABLE_SIMD options, compiler cache)</t>
+  </si>
+  <si>
+    <t>yes (performance-focused changes documented in changelog)</t>
+  </si>
+  <si>
+    <t>yes (VAMP integration with SIMD, build type options for Release/RelWithDebInfo, parallel builds)</t>
+  </si>
+  <si>
+    <t>yes (benchmark infrastructure, tracy profiler option, CRTP pattern mentioned)</t>
+  </si>
+  <si>
+    <t>yes (parallel execution options, performance optimizations mentioned)</t>
+  </si>
+  <si>
+    <t>yes (SSE/AVX/GPU solver options, parallel processing, caching)</t>
+  </si>
+  <si>
+    <r>
+      <t>Is there evidence that performance was considered? Performance refers to either speed, storage, or throughput. (yes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Cambria Math"/>
+        <family val="1"/>
+      </rPr>
+      <t>∗</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, no)</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2279,6 +2254,20 @@
       <sz val="11"/>
       <name val="Cambria Math"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Cambria Math"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -4096,7 +4085,7 @@
         <v>167</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>481</v>
+        <v>455</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>168</v>
@@ -6533,93 +6522,93 @@
       </c>
       <c r="AD48" s="3"/>
     </row>
-    <row r="49" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>430</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="H49" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="I49" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="J49" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="K49" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="L49" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="M49" s="1" t="s">
-        <v>436</v>
-      </c>
-      <c r="N49" s="1" t="s">
-        <v>437</v>
-      </c>
-      <c r="O49" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="P49" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="Q49" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="R49" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="S49" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="T49" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="U49" s="1" t="s">
-        <v>444</v>
-      </c>
-      <c r="V49" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="W49" s="1" t="s">
-        <v>446</v>
-      </c>
-      <c r="X49" s="1" t="s">
-        <v>447</v>
-      </c>
-      <c r="Y49" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="Z49" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="AA49" s="1" t="s">
-        <v>450</v>
-      </c>
-      <c r="AB49" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="AC49" s="1" t="s">
-        <v>452</v>
+    <row r="49" spans="1:30" customFormat="1" ht="86.15" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>674</v>
+      </c>
+      <c r="B49" t="s">
+        <v>665</v>
+      </c>
+      <c r="C49" t="s">
+        <v>665</v>
+      </c>
+      <c r="D49" t="s">
+        <v>665</v>
+      </c>
+      <c r="E49" t="s">
+        <v>665</v>
+      </c>
+      <c r="F49" t="s">
+        <v>665</v>
+      </c>
+      <c r="G49" t="s">
+        <v>665</v>
+      </c>
+      <c r="H49" t="s">
+        <v>665</v>
+      </c>
+      <c r="I49" t="s">
+        <v>666</v>
+      </c>
+      <c r="J49" t="s">
+        <v>667</v>
+      </c>
+      <c r="K49" t="s">
+        <v>665</v>
+      </c>
+      <c r="L49" t="s">
+        <v>665</v>
+      </c>
+      <c r="M49" t="s">
+        <v>668</v>
+      </c>
+      <c r="N49" t="s">
+        <v>669</v>
+      </c>
+      <c r="O49" t="s">
+        <v>665</v>
+      </c>
+      <c r="P49" t="s">
+        <v>665</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>670</v>
+      </c>
+      <c r="R49" t="s">
+        <v>671</v>
+      </c>
+      <c r="S49" t="s">
+        <v>665</v>
+      </c>
+      <c r="T49" t="s">
+        <v>672</v>
+      </c>
+      <c r="U49" t="s">
+        <v>665</v>
+      </c>
+      <c r="V49" t="s">
+        <v>665</v>
+      </c>
+      <c r="W49" t="s">
+        <v>665</v>
+      </c>
+      <c r="X49" t="s">
+        <v>665</v>
+      </c>
+      <c r="Y49" t="s">
+        <v>665</v>
+      </c>
+      <c r="Z49" t="s">
+        <v>665</v>
+      </c>
+      <c r="AA49" t="s">
+        <v>673</v>
+      </c>
+      <c r="AB49" t="s">
+        <v>665</v>
+      </c>
+      <c r="AC49" t="s">
+        <v>665</v>
       </c>
     </row>
     <row r="50" spans="1:30" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
@@ -8279,91 +8268,91 @@
     </row>
     <row r="77" spans="1:30" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A77" s="17" t="s">
-        <v>480</v>
+        <v>454</v>
       </c>
       <c r="B77" s="17" t="s">
-        <v>453</v>
+        <v>427</v>
       </c>
       <c r="C77" s="17" t="s">
-        <v>454</v>
+        <v>428</v>
       </c>
       <c r="D77" s="17" t="s">
-        <v>455</v>
+        <v>429</v>
       </c>
       <c r="E77" s="17" t="s">
-        <v>456</v>
+        <v>430</v>
       </c>
       <c r="F77" s="17" t="s">
-        <v>457</v>
+        <v>431</v>
       </c>
       <c r="G77" s="1" t="s">
         <v>131</v>
       </c>
       <c r="H77" s="17" t="s">
-        <v>458</v>
+        <v>432</v>
       </c>
       <c r="I77" s="17" t="s">
-        <v>459</v>
+        <v>433</v>
       </c>
       <c r="J77" s="17" t="s">
-        <v>460</v>
+        <v>434</v>
       </c>
       <c r="K77" s="17" t="s">
-        <v>461</v>
+        <v>435</v>
       </c>
       <c r="L77" s="17" t="s">
-        <v>462</v>
+        <v>436</v>
       </c>
       <c r="M77" s="17" t="s">
-        <v>463</v>
+        <v>437</v>
       </c>
       <c r="N77" s="17" t="s">
-        <v>464</v>
+        <v>438</v>
       </c>
       <c r="O77" s="17" t="s">
-        <v>465</v>
+        <v>439</v>
       </c>
       <c r="P77" s="17" t="s">
-        <v>466</v>
+        <v>440</v>
       </c>
       <c r="Q77" s="17" t="s">
-        <v>467</v>
+        <v>441</v>
       </c>
       <c r="R77" s="17" t="s">
-        <v>468</v>
+        <v>442</v>
       </c>
       <c r="S77" s="17" t="s">
-        <v>469</v>
+        <v>443</v>
       </c>
       <c r="T77" s="17" t="s">
-        <v>470</v>
+        <v>444</v>
       </c>
       <c r="U77" s="17" t="s">
-        <v>471</v>
+        <v>445</v>
       </c>
       <c r="V77" s="17" t="s">
-        <v>472</v>
+        <v>446</v>
       </c>
       <c r="W77" s="17" t="s">
-        <v>473</v>
+        <v>447</v>
       </c>
       <c r="X77" s="17" t="s">
-        <v>474</v>
+        <v>448</v>
       </c>
       <c r="Y77" s="17" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="Z77" s="17" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="AA77" s="17" t="s">
-        <v>477</v>
+        <v>451</v>
       </c>
       <c r="AB77" s="17" t="s">
-        <v>478</v>
+        <v>452</v>
       </c>
       <c r="AC77" s="17" t="s">
-        <v>479</v>
+        <v>453</v>
       </c>
     </row>
     <row r="78" spans="1:30" ht="42.45" customHeight="1" x14ac:dyDescent="0.35">
@@ -8458,91 +8447,91 @@
     </row>
     <row r="79" spans="1:30" s="17" customFormat="1" ht="70.75" x14ac:dyDescent="0.35">
       <c r="A79" s="17" t="s">
+        <v>456</v>
+      </c>
+      <c r="B79" s="17" t="s">
+        <v>457</v>
+      </c>
+      <c r="C79" s="17" t="s">
+        <v>458</v>
+      </c>
+      <c r="D79" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="E79" s="17" t="s">
+        <v>460</v>
+      </c>
+      <c r="F79" s="17" t="s">
+        <v>461</v>
+      </c>
+      <c r="G79" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="H79" s="17" t="s">
+        <v>463</v>
+      </c>
+      <c r="I79" s="17" t="s">
+        <v>464</v>
+      </c>
+      <c r="J79" s="17" t="s">
+        <v>465</v>
+      </c>
+      <c r="K79" s="17" t="s">
+        <v>466</v>
+      </c>
+      <c r="L79" s="17" t="s">
+        <v>467</v>
+      </c>
+      <c r="M79" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="N79" s="17" t="s">
+        <v>469</v>
+      </c>
+      <c r="O79" s="17" t="s">
+        <v>470</v>
+      </c>
+      <c r="P79" s="17" t="s">
+        <v>471</v>
+      </c>
+      <c r="Q79" s="17" t="s">
+        <v>472</v>
+      </c>
+      <c r="R79" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="S79" s="17" t="s">
+        <v>474</v>
+      </c>
+      <c r="T79" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="U79" s="17" t="s">
+        <v>476</v>
+      </c>
+      <c r="V79" s="17" t="s">
+        <v>477</v>
+      </c>
+      <c r="W79" s="17" t="s">
+        <v>478</v>
+      </c>
+      <c r="X79" s="17" t="s">
+        <v>479</v>
+      </c>
+      <c r="Y79" s="17" t="s">
+        <v>480</v>
+      </c>
+      <c r="Z79" s="17" t="s">
+        <v>481</v>
+      </c>
+      <c r="AA79" s="17" t="s">
         <v>482</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="AB79" s="17" t="s">
         <v>483</v>
       </c>
-      <c r="C79" s="17" t="s">
+      <c r="AC79" s="17" t="s">
         <v>484</v>
-      </c>
-      <c r="D79" s="17" t="s">
-        <v>485</v>
-      </c>
-      <c r="E79" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="F79" s="17" t="s">
-        <v>487</v>
-      </c>
-      <c r="G79" s="17" t="s">
-        <v>488</v>
-      </c>
-      <c r="H79" s="17" t="s">
-        <v>489</v>
-      </c>
-      <c r="I79" s="17" t="s">
-        <v>490</v>
-      </c>
-      <c r="J79" s="17" t="s">
-        <v>491</v>
-      </c>
-      <c r="K79" s="17" t="s">
-        <v>492</v>
-      </c>
-      <c r="L79" s="17" t="s">
-        <v>493</v>
-      </c>
-      <c r="M79" s="17" t="s">
-        <v>494</v>
-      </c>
-      <c r="N79" s="17" t="s">
-        <v>495</v>
-      </c>
-      <c r="O79" s="17" t="s">
-        <v>496</v>
-      </c>
-      <c r="P79" s="17" t="s">
-        <v>497</v>
-      </c>
-      <c r="Q79" s="17" t="s">
-        <v>498</v>
-      </c>
-      <c r="R79" s="17" t="s">
-        <v>499</v>
-      </c>
-      <c r="S79" s="17" t="s">
-        <v>500</v>
-      </c>
-      <c r="T79" s="17" t="s">
-        <v>501</v>
-      </c>
-      <c r="U79" s="17" t="s">
-        <v>502</v>
-      </c>
-      <c r="V79" s="17" t="s">
-        <v>503</v>
-      </c>
-      <c r="W79" s="17" t="s">
-        <v>504</v>
-      </c>
-      <c r="X79" s="17" t="s">
-        <v>505</v>
-      </c>
-      <c r="Y79" s="17" t="s">
-        <v>506</v>
-      </c>
-      <c r="Z79" s="17" t="s">
-        <v>507</v>
-      </c>
-      <c r="AA79" s="17" t="s">
-        <v>508</v>
-      </c>
-      <c r="AB79" s="17" t="s">
-        <v>509</v>
-      </c>
-      <c r="AC79" s="17" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="80" spans="1:30" ht="84.9" customHeight="1" x14ac:dyDescent="0.35">
@@ -8637,180 +8626,180 @@
     </row>
     <row r="81" spans="1:30" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A81" s="17" t="s">
-        <v>511</v>
+        <v>485</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>512</v>
+        <v>486</v>
       </c>
       <c r="C81" s="17" t="s">
-        <v>513</v>
+        <v>487</v>
       </c>
       <c r="D81" s="17" t="s">
-        <v>514</v>
+        <v>488</v>
       </c>
       <c r="E81" s="17" t="s">
-        <v>515</v>
+        <v>489</v>
       </c>
       <c r="F81" s="17" t="s">
-        <v>516</v>
+        <v>490</v>
       </c>
       <c r="G81" s="17" t="s">
         <v>76</v>
       </c>
       <c r="H81" s="17" t="s">
-        <v>517</v>
+        <v>491</v>
       </c>
       <c r="I81" s="17" t="s">
-        <v>518</v>
+        <v>492</v>
       </c>
       <c r="J81" s="17" t="s">
-        <v>519</v>
+        <v>493</v>
       </c>
       <c r="K81" s="17" t="s">
-        <v>520</v>
+        <v>494</v>
       </c>
       <c r="L81" s="17" t="s">
-        <v>521</v>
+        <v>495</v>
       </c>
       <c r="M81" s="17" t="s">
-        <v>522</v>
+        <v>496</v>
       </c>
       <c r="N81" s="17" t="s">
-        <v>523</v>
+        <v>497</v>
       </c>
       <c r="O81" s="17" t="s">
-        <v>524</v>
+        <v>498</v>
       </c>
       <c r="P81" s="17" t="s">
-        <v>525</v>
+        <v>499</v>
       </c>
       <c r="Q81" s="17" t="s">
-        <v>526</v>
+        <v>500</v>
       </c>
       <c r="R81" s="17" t="s">
-        <v>527</v>
+        <v>501</v>
       </c>
       <c r="S81" s="17" t="s">
-        <v>528</v>
+        <v>502</v>
       </c>
       <c r="T81" s="17" t="s">
-        <v>529</v>
+        <v>503</v>
       </c>
       <c r="U81" s="17" t="s">
-        <v>530</v>
+        <v>504</v>
       </c>
       <c r="V81" s="17" t="s">
-        <v>531</v>
+        <v>505</v>
       </c>
       <c r="W81" s="17" t="s">
-        <v>532</v>
+        <v>506</v>
       </c>
       <c r="X81" s="17" t="s">
-        <v>533</v>
+        <v>507</v>
       </c>
       <c r="Y81" s="17" t="s">
-        <v>534</v>
+        <v>508</v>
       </c>
       <c r="Z81" s="17" t="s">
-        <v>535</v>
+        <v>509</v>
       </c>
       <c r="AA81" s="17" t="s">
-        <v>522</v>
+        <v>496</v>
       </c>
       <c r="AB81" s="17" t="s">
-        <v>536</v>
+        <v>510</v>
       </c>
       <c r="AC81" s="17" t="s">
-        <v>537</v>
+        <v>511</v>
       </c>
     </row>
     <row r="82" spans="1:30" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A82" s="17" t="s">
+        <v>512</v>
+      </c>
+      <c r="B82" s="17" t="s">
+        <v>513</v>
+      </c>
+      <c r="C82" s="17" t="s">
+        <v>514</v>
+      </c>
+      <c r="D82" s="17" t="s">
+        <v>515</v>
+      </c>
+      <c r="E82" s="17" t="s">
+        <v>516</v>
+      </c>
+      <c r="F82" s="17" t="s">
+        <v>517</v>
+      </c>
+      <c r="G82" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="H82" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="I82" s="17" t="s">
+        <v>520</v>
+      </c>
+      <c r="J82" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="K82" s="17" t="s">
+        <v>522</v>
+      </c>
+      <c r="L82" s="17" t="s">
+        <v>523</v>
+      </c>
+      <c r="M82" s="17" t="s">
+        <v>524</v>
+      </c>
+      <c r="N82" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="O82" s="17" t="s">
+        <v>526</v>
+      </c>
+      <c r="P82" s="17" t="s">
+        <v>527</v>
+      </c>
+      <c r="Q82" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="R82" s="17" t="s">
+        <v>529</v>
+      </c>
+      <c r="S82" s="17" t="s">
+        <v>530</v>
+      </c>
+      <c r="T82" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="U82" s="17" t="s">
+        <v>532</v>
+      </c>
+      <c r="V82" s="17" t="s">
+        <v>533</v>
+      </c>
+      <c r="W82" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="X82" s="17" t="s">
+        <v>535</v>
+      </c>
+      <c r="Y82" s="17" t="s">
+        <v>536</v>
+      </c>
+      <c r="Z82" s="17" t="s">
+        <v>537</v>
+      </c>
+      <c r="AA82" s="17" t="s">
         <v>538</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="AB82" s="17" t="s">
         <v>539</v>
       </c>
-      <c r="C82" s="17" t="s">
+      <c r="AC82" s="17" t="s">
         <v>540</v>
-      </c>
-      <c r="D82" s="17" t="s">
-        <v>541</v>
-      </c>
-      <c r="E82" s="17" t="s">
-        <v>542</v>
-      </c>
-      <c r="F82" s="17" t="s">
-        <v>543</v>
-      </c>
-      <c r="G82" s="17" t="s">
-        <v>544</v>
-      </c>
-      <c r="H82" s="17" t="s">
-        <v>545</v>
-      </c>
-      <c r="I82" s="17" t="s">
-        <v>546</v>
-      </c>
-      <c r="J82" s="17" t="s">
-        <v>547</v>
-      </c>
-      <c r="K82" s="17" t="s">
-        <v>548</v>
-      </c>
-      <c r="L82" s="17" t="s">
-        <v>549</v>
-      </c>
-      <c r="M82" s="17" t="s">
-        <v>550</v>
-      </c>
-      <c r="N82" s="17" t="s">
-        <v>551</v>
-      </c>
-      <c r="O82" s="17" t="s">
-        <v>552</v>
-      </c>
-      <c r="P82" s="17" t="s">
-        <v>553</v>
-      </c>
-      <c r="Q82" s="17" t="s">
-        <v>554</v>
-      </c>
-      <c r="R82" s="17" t="s">
-        <v>555</v>
-      </c>
-      <c r="S82" s="17" t="s">
-        <v>556</v>
-      </c>
-      <c r="T82" s="17" t="s">
-        <v>557</v>
-      </c>
-      <c r="U82" s="17" t="s">
-        <v>558</v>
-      </c>
-      <c r="V82" s="17" t="s">
-        <v>559</v>
-      </c>
-      <c r="W82" s="17" t="s">
-        <v>560</v>
-      </c>
-      <c r="X82" s="17" t="s">
-        <v>561</v>
-      </c>
-      <c r="Y82" s="17" t="s">
-        <v>562</v>
-      </c>
-      <c r="Z82" s="17" t="s">
-        <v>563</v>
-      </c>
-      <c r="AA82" s="17" t="s">
-        <v>564</v>
-      </c>
-      <c r="AB82" s="17" t="s">
-        <v>565</v>
-      </c>
-      <c r="AC82" s="17" t="s">
-        <v>566</v>
       </c>
     </row>
     <row r="83" spans="1:30" ht="56.6" customHeight="1" x14ac:dyDescent="0.35">
@@ -9098,91 +9087,91 @@
     </row>
     <row r="89" spans="1:30" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A89" s="17" t="s">
+        <v>541</v>
+      </c>
+      <c r="B89" s="17" t="s">
+        <v>542</v>
+      </c>
+      <c r="C89" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="D89" s="17" t="s">
+        <v>544</v>
+      </c>
+      <c r="E89" s="17" t="s">
+        <v>545</v>
+      </c>
+      <c r="F89" s="17" t="s">
+        <v>546</v>
+      </c>
+      <c r="G89" s="17" t="s">
+        <v>547</v>
+      </c>
+      <c r="H89" s="17" t="s">
+        <v>548</v>
+      </c>
+      <c r="I89" s="17" t="s">
+        <v>549</v>
+      </c>
+      <c r="J89" s="17" t="s">
+        <v>550</v>
+      </c>
+      <c r="K89" s="17" t="s">
+        <v>551</v>
+      </c>
+      <c r="L89" s="17" t="s">
+        <v>552</v>
+      </c>
+      <c r="M89" s="17" t="s">
+        <v>553</v>
+      </c>
+      <c r="N89" s="17" t="s">
+        <v>554</v>
+      </c>
+      <c r="O89" s="17" t="s">
+        <v>555</v>
+      </c>
+      <c r="P89" s="17" t="s">
+        <v>556</v>
+      </c>
+      <c r="Q89" s="17" t="s">
+        <v>557</v>
+      </c>
+      <c r="R89" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="S89" s="17" t="s">
+        <v>559</v>
+      </c>
+      <c r="T89" s="17" t="s">
+        <v>560</v>
+      </c>
+      <c r="U89" s="17" t="s">
+        <v>561</v>
+      </c>
+      <c r="V89" s="17" t="s">
+        <v>562</v>
+      </c>
+      <c r="W89" s="17" t="s">
+        <v>563</v>
+      </c>
+      <c r="X89" s="17" t="s">
+        <v>564</v>
+      </c>
+      <c r="Y89" s="17" t="s">
+        <v>565</v>
+      </c>
+      <c r="Z89" s="17" t="s">
+        <v>566</v>
+      </c>
+      <c r="AA89" s="17" t="s">
         <v>567</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="AB89" s="17" t="s">
         <v>568</v>
       </c>
-      <c r="C89" s="17" t="s">
+      <c r="AC89" s="17" t="s">
         <v>569</v>
-      </c>
-      <c r="D89" s="17" t="s">
-        <v>570</v>
-      </c>
-      <c r="E89" s="17" t="s">
-        <v>571</v>
-      </c>
-      <c r="F89" s="17" t="s">
-        <v>572</v>
-      </c>
-      <c r="G89" s="17" t="s">
-        <v>573</v>
-      </c>
-      <c r="H89" s="17" t="s">
-        <v>574</v>
-      </c>
-      <c r="I89" s="17" t="s">
-        <v>575</v>
-      </c>
-      <c r="J89" s="17" t="s">
-        <v>576</v>
-      </c>
-      <c r="K89" s="17" t="s">
-        <v>577</v>
-      </c>
-      <c r="L89" s="17" t="s">
-        <v>578</v>
-      </c>
-      <c r="M89" s="17" t="s">
-        <v>579</v>
-      </c>
-      <c r="N89" s="17" t="s">
-        <v>580</v>
-      </c>
-      <c r="O89" s="17" t="s">
-        <v>581</v>
-      </c>
-      <c r="P89" s="17" t="s">
-        <v>582</v>
-      </c>
-      <c r="Q89" s="17" t="s">
-        <v>583</v>
-      </c>
-      <c r="R89" s="17" t="s">
-        <v>584</v>
-      </c>
-      <c r="S89" s="17" t="s">
-        <v>585</v>
-      </c>
-      <c r="T89" s="17" t="s">
-        <v>586</v>
-      </c>
-      <c r="U89" s="17" t="s">
-        <v>587</v>
-      </c>
-      <c r="V89" s="17" t="s">
-        <v>588</v>
-      </c>
-      <c r="W89" s="17" t="s">
-        <v>589</v>
-      </c>
-      <c r="X89" s="17" t="s">
-        <v>590</v>
-      </c>
-      <c r="Y89" s="17" t="s">
-        <v>591</v>
-      </c>
-      <c r="Z89" s="17" t="s">
-        <v>592</v>
-      </c>
-      <c r="AA89" s="17" t="s">
-        <v>593</v>
-      </c>
-      <c r="AB89" s="17" t="s">
-        <v>594</v>
-      </c>
-      <c r="AC89" s="17" t="s">
-        <v>595</v>
       </c>
     </row>
     <row r="90" spans="1:30" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
@@ -10319,91 +10308,91 @@
     </row>
     <row r="109" spans="1:30" s="17" customFormat="1" ht="28.3" x14ac:dyDescent="0.35">
       <c r="A109" s="17" t="s">
-        <v>596</v>
+        <v>570</v>
       </c>
       <c r="B109" s="17" t="s">
-        <v>597</v>
+        <v>571</v>
       </c>
       <c r="C109" s="17" t="s">
-        <v>598</v>
+        <v>572</v>
       </c>
       <c r="D109" s="17" t="s">
-        <v>599</v>
+        <v>573</v>
       </c>
       <c r="E109" s="17" t="s">
         <v>131</v>
       </c>
       <c r="F109" s="17" t="s">
-        <v>600</v>
+        <v>574</v>
       </c>
       <c r="G109" s="17" t="s">
         <v>131</v>
       </c>
       <c r="H109" s="17" t="s">
-        <v>601</v>
+        <v>575</v>
       </c>
       <c r="I109" s="17" t="s">
-        <v>602</v>
+        <v>576</v>
       </c>
       <c r="J109" s="17" t="s">
-        <v>603</v>
+        <v>577</v>
       </c>
       <c r="K109" s="17" t="s">
-        <v>604</v>
+        <v>578</v>
       </c>
       <c r="L109" s="17" t="s">
-        <v>605</v>
+        <v>579</v>
       </c>
       <c r="M109" s="17" t="s">
-        <v>606</v>
+        <v>580</v>
       </c>
       <c r="N109" s="17" t="s">
-        <v>607</v>
+        <v>581</v>
       </c>
       <c r="O109" s="17" t="s">
-        <v>608</v>
+        <v>582</v>
       </c>
       <c r="P109" s="17" t="s">
-        <v>609</v>
+        <v>583</v>
       </c>
       <c r="Q109" s="17" t="s">
         <v>131</v>
       </c>
       <c r="R109" s="17" t="s">
-        <v>610</v>
+        <v>584</v>
       </c>
       <c r="S109" s="17" t="s">
-        <v>611</v>
+        <v>585</v>
       </c>
       <c r="T109" s="17" t="s">
-        <v>612</v>
+        <v>586</v>
       </c>
       <c r="U109" s="17" t="s">
-        <v>613</v>
+        <v>587</v>
       </c>
       <c r="V109" s="17" t="s">
-        <v>614</v>
+        <v>588</v>
       </c>
       <c r="W109" s="17" t="s">
-        <v>615</v>
+        <v>589</v>
       </c>
       <c r="X109" s="17" t="s">
-        <v>616</v>
+        <v>590</v>
       </c>
       <c r="Y109" s="17" t="s">
-        <v>617</v>
+        <v>591</v>
       </c>
       <c r="Z109" s="17" t="s">
-        <v>618</v>
+        <v>592</v>
       </c>
       <c r="AA109" s="17" t="s">
-        <v>619</v>
+        <v>593</v>
       </c>
       <c r="AB109" s="17" t="s">
-        <v>620</v>
+        <v>594</v>
       </c>
       <c r="AC109" s="17" t="s">
-        <v>621</v>
+        <v>595</v>
       </c>
     </row>
     <row r="110" spans="1:30" ht="42.45" customHeight="1" x14ac:dyDescent="0.35">
@@ -10906,7 +10895,7 @@
     </row>
     <row r="119" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>622</v>
+        <v>596</v>
       </c>
       <c r="B119">
         <v>1765</v>
@@ -11000,7 +10989,7 @@
     </row>
     <row r="120" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>623</v>
+        <v>597</v>
       </c>
       <c r="B120">
         <v>210</v>
@@ -11094,7 +11083,7 @@
     </row>
     <row r="121" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>624</v>
+        <v>598</v>
       </c>
       <c r="B121">
         <v>704551</v>
@@ -11188,7 +11177,7 @@
     </row>
     <row r="122" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>625</v>
+        <v>599</v>
       </c>
       <c r="B122">
         <v>1460745</v>
@@ -11282,7 +11271,7 @@
     </row>
     <row r="123" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>626</v>
+        <v>600</v>
       </c>
       <c r="B123">
         <v>691522</v>
@@ -11376,7 +11365,7 @@
     </row>
     <row r="124" spans="1:34" ht="56.6" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>627</v>
+        <v>601</v>
       </c>
       <c r="B124">
         <v>7500</v>
@@ -11468,197 +11457,187 @@
       <c r="AG124"/>
       <c r="AH124"/>
     </row>
-    <row r="125" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:34" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
+        <v>602</v>
+      </c>
+      <c r="B125" t="s">
+        <v>612</v>
+      </c>
+      <c r="C125" t="s">
+        <v>613</v>
+      </c>
+      <c r="D125" t="s">
+        <v>614</v>
+      </c>
+      <c r="E125" t="s">
+        <v>615</v>
+      </c>
+      <c r="F125" t="s">
+        <v>616</v>
+      </c>
+      <c r="G125" t="s">
+        <v>617</v>
+      </c>
+      <c r="H125" t="s">
+        <v>618</v>
+      </c>
+      <c r="I125" t="s">
+        <v>619</v>
+      </c>
+      <c r="J125" t="s">
+        <v>620</v>
+      </c>
+      <c r="K125" t="s">
+        <v>621</v>
+      </c>
+      <c r="L125" t="s">
+        <v>622</v>
+      </c>
+      <c r="M125" t="s">
+        <v>623</v>
+      </c>
+      <c r="N125" t="s">
+        <v>624</v>
+      </c>
+      <c r="O125" t="s">
+        <v>625</v>
+      </c>
+      <c r="P125" t="s">
+        <v>626</v>
+      </c>
+      <c r="Q125" t="s">
+        <v>627</v>
+      </c>
+      <c r="R125" t="s">
         <v>628</v>
       </c>
-      <c r="B125" t="s">
+      <c r="S125" t="s">
         <v>629</v>
       </c>
-      <c r="C125" t="s">
+      <c r="T125" t="s">
         <v>630</v>
       </c>
-      <c r="D125" t="s">
+      <c r="U125" t="s">
         <v>631</v>
       </c>
-      <c r="E125" t="s">
+      <c r="V125" t="s">
         <v>632</v>
       </c>
-      <c r="F125" t="s">
+      <c r="W125" t="s">
         <v>633</v>
       </c>
-      <c r="G125" t="s">
+      <c r="X125" t="s">
         <v>634</v>
       </c>
-      <c r="H125" t="s">
+      <c r="Y125" t="s">
         <v>635</v>
       </c>
-      <c r="I125" t="s">
+      <c r="Z125" t="s">
         <v>636</v>
       </c>
-      <c r="J125" t="s">
+      <c r="AA125" t="s">
         <v>637</v>
       </c>
-      <c r="K125" t="s">
+      <c r="AB125" t="s">
         <v>638</v>
       </c>
-      <c r="L125" t="s">
+      <c r="AC125" t="s">
         <v>639</v>
       </c>
-      <c r="M125" t="s">
+    </row>
+    <row r="126" spans="1:34" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>603</v>
+      </c>
+      <c r="B126" t="s">
         <v>640</v>
       </c>
-      <c r="N125" t="s">
+      <c r="C126" t="s">
         <v>641</v>
       </c>
-      <c r="O125" t="s">
+      <c r="D126" t="s">
         <v>642</v>
       </c>
-      <c r="P125" t="s">
+      <c r="E126" t="s">
         <v>643</v>
       </c>
-      <c r="Q125" t="s">
+      <c r="F126" t="s">
         <v>644</v>
       </c>
-      <c r="R125" t="s">
+      <c r="G126" t="s">
         <v>645</v>
       </c>
-      <c r="S125" t="s">
+      <c r="H126" t="s">
         <v>646</v>
       </c>
-      <c r="T125" t="s">
+      <c r="I126" t="s">
         <v>647</v>
       </c>
-      <c r="U125" t="s">
+      <c r="J126" t="s">
         <v>648</v>
       </c>
-      <c r="V125" t="s">
+      <c r="K126" t="s">
         <v>649</v>
       </c>
-      <c r="W125" t="s">
+      <c r="L126" t="s">
         <v>650</v>
       </c>
-      <c r="X125" t="s">
+      <c r="M126" t="s">
         <v>651</v>
       </c>
-      <c r="Y125" t="s">
+      <c r="N126" t="s">
         <v>652</v>
       </c>
-      <c r="Z125" t="s">
+      <c r="O126" t="s">
+        <v>647</v>
+      </c>
+      <c r="P126" t="s">
         <v>653</v>
       </c>
-      <c r="AA125" t="s">
+      <c r="Q126" t="s">
         <v>654</v>
       </c>
-      <c r="AB125" t="s">
+      <c r="R126" t="s">
         <v>655</v>
       </c>
-      <c r="AC125" t="s">
+      <c r="S126" t="s">
         <v>656</v>
       </c>
-      <c r="AD125"/>
-      <c r="AE125"/>
-      <c r="AF125"/>
-      <c r="AG125"/>
-      <c r="AH125"/>
-    </row>
-    <row r="126" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A126" t="s">
+      <c r="T126" t="s">
         <v>657</v>
       </c>
-      <c r="B126" t="s">
+      <c r="U126" t="s">
         <v>658</v>
       </c>
-      <c r="C126" t="s">
+      <c r="V126" t="s">
+        <v>647</v>
+      </c>
+      <c r="W126" t="s">
         <v>659</v>
       </c>
-      <c r="D126" t="s">
+      <c r="X126" t="s">
         <v>660</v>
       </c>
-      <c r="E126" t="s">
+      <c r="Y126" t="s">
+        <v>647</v>
+      </c>
+      <c r="Z126" t="s">
         <v>661</v>
       </c>
-      <c r="F126" t="s">
+      <c r="AA126" t="s">
         <v>662</v>
       </c>
-      <c r="G126" t="s">
+      <c r="AB126" t="s">
         <v>663</v>
       </c>
-      <c r="H126" t="s">
+      <c r="AC126" t="s">
         <v>664</v>
       </c>
-      <c r="I126" t="s">
-        <v>665</v>
-      </c>
-      <c r="J126" t="s">
-        <v>666</v>
-      </c>
-      <c r="K126" t="s">
-        <v>667</v>
-      </c>
-      <c r="L126" t="s">
-        <v>668</v>
-      </c>
-      <c r="M126" t="s">
-        <v>669</v>
-      </c>
-      <c r="N126" t="s">
-        <v>670</v>
-      </c>
-      <c r="O126" t="s">
-        <v>665</v>
-      </c>
-      <c r="P126" t="s">
-        <v>671</v>
-      </c>
-      <c r="Q126" t="s">
-        <v>672</v>
-      </c>
-      <c r="R126" t="s">
-        <v>673</v>
-      </c>
-      <c r="S126" t="s">
-        <v>674</v>
-      </c>
-      <c r="T126" t="s">
-        <v>675</v>
-      </c>
-      <c r="U126" t="s">
-        <v>676</v>
-      </c>
-      <c r="V126" t="s">
-        <v>665</v>
-      </c>
-      <c r="W126" t="s">
-        <v>677</v>
-      </c>
-      <c r="X126" t="s">
-        <v>678</v>
-      </c>
-      <c r="Y126" t="s">
-        <v>665</v>
-      </c>
-      <c r="Z126" t="s">
-        <v>679</v>
-      </c>
-      <c r="AA126" t="s">
-        <v>680</v>
-      </c>
-      <c r="AB126" t="s">
-        <v>681</v>
-      </c>
-      <c r="AC126" t="s">
-        <v>682</v>
-      </c>
-      <c r="AD126"/>
-      <c r="AE126"/>
-      <c r="AF126"/>
-      <c r="AG126"/>
-      <c r="AH126"/>
     </row>
     <row r="127" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>622</v>
+        <v>596</v>
       </c>
       <c r="B127">
         <v>1765</v>
@@ -11752,7 +11731,7 @@
     </row>
     <row r="128" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>624</v>
+        <v>598</v>
       </c>
       <c r="B128">
         <v>704551</v>
@@ -11846,7 +11825,7 @@
     </row>
     <row r="129" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>683</v>
+        <v>604</v>
       </c>
       <c r="B129">
         <v>193808</v>
@@ -11940,7 +11919,7 @@
     </row>
     <row r="130" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>684</v>
+        <v>605</v>
       </c>
       <c r="B130">
         <v>83838</v>
@@ -12034,7 +12013,7 @@
     </row>
     <row r="131" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>685</v>
+        <v>606</v>
       </c>
       <c r="B131">
         <v>77856</v>
@@ -12128,7 +12107,7 @@
     </row>
     <row r="132" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>686</v>
+        <v>607</v>
       </c>
       <c r="B132">
         <v>1337</v>
@@ -12222,7 +12201,7 @@
     </row>
     <row r="133" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>687</v>
+        <v>608</v>
       </c>
       <c r="B133">
         <v>411</v>
@@ -12316,7 +12295,7 @@
     </row>
     <row r="134" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>688</v>
+        <v>609</v>
       </c>
       <c r="B134">
         <v>22</v>
@@ -12410,7 +12389,7 @@
     </row>
     <row r="135" spans="1:34" ht="28.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>689</v>
+        <v>610</v>
       </c>
       <c r="B135">
         <v>92</v>
@@ -12504,7 +12483,7 @@
     </row>
     <row r="136" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>690</v>
+        <v>611</v>
       </c>
       <c r="B136">
         <v>2358</v>

</xml_diff>